<commit_message>
Actualización Tablero CUN - 03/08/2026 04:27 PM
</commit_message>
<xml_diff>
--- a/Facilitadores_Pendientes_Asistencia.xlsx
+++ b/Facilitadores_Pendientes_Asistencia.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U331"/>
+  <dimension ref="A1:U332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -32510,6 +32510,75 @@
         <v/>
       </c>
     </row>
+    <row r="332" ht="20" customHeight="1">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
+      </c>
+      <c r="B332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="C332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="D332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="E332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="F332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="G332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="H332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="I332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="J332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="K332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="L332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="M332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="N332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="O332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="P332" s="3" t="inlineStr">
+        <is>
+          <t>CONFIRMADO VIRTUAL</t>
+        </is>
+      </c>
+      <c r="Q332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="R332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="S332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="T332" s="3" t="n">
+        <v/>
+      </c>
+      <c r="U332" s="3" t="n">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>